<commit_message>
deployed Framworks/ivbox and implemented scrapping sofascore
</commit_message>
<xml_diff>
--- a/webscrapping/sofascore/files_initted/jornadas_info_db.xlsx
+++ b/webscrapping/sofascore/files_initted/jornadas_info_db.xlsx
@@ -14,12 +14,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>id_jornada</t>
   </si>
   <si>
     <t>id_temporada</t>
+  </si>
+  <si>
+    <t>fecha_creacion</t>
   </si>
 </sst>
 </file>
@@ -377,127 +380,172 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:2">
+      <c r="C2">
+        <v>1765192183</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:2">
+      <c r="C3">
+        <v>1765192183</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:2">
+      <c r="C4">
+        <v>1765192183</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:2">
+      <c r="C5">
+        <v>1765192183</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:2">
+      <c r="C6">
+        <v>1765192183</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:2">
+      <c r="C7">
+        <v>1765192183</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:2">
+      <c r="C8">
+        <v>1765192183</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:2">
+      <c r="C9">
+        <v>1765192183</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:2">
+      <c r="C10">
+        <v>1765192183</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:2">
+      <c r="C11">
+        <v>1765192183</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:2">
+      <c r="C12">
+        <v>1765192183</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:2">
+      <c r="C13">
+        <v>1765192183</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:2">
+      <c r="C14">
+        <v>1765192183</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15">
         <v>1</v>
+      </c>
+      <c r="C15">
+        <v>1765192183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>